<commit_message>
dr-aliabadi: round 6 corrections
Workbook Read Me pillar split corrected (it kept a pre-rebuild 47/24/17/16/16
that still summed to 120, so nothing caught it). Slide 13's endometriosis card
no longer reads '17 articles' above 'Held at sixteen'. Slide 6's surgery row
drops a URL count no source produced and states the 18 procedure pages she
actually has.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/dr-aliabadi/keyword-research.xlsx
+++ b/decks/dr-aliabadi/keyword-research.xlsx
@@ -1349,8 +1349,10 @@
       <c r="G14" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="H14" s="15" t="n">
-        <v>0</v>
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1558,8 +1560,10 @@
       <c r="G18" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="H18" s="15" t="n">
-        <v>0</v>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -2241,8 +2245,10 @@
       <c r="G31" s="4" t="n">
         <v>720</v>
       </c>
-      <c r="H31" s="15" t="n">
-        <v>0</v>
+      <c r="H31" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -5489,8 +5495,10 @@
       <c r="G94" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="H94" s="15" t="n">
-        <v>0</v>
+      <c r="H94" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
@@ -17799,8 +17807,10 @@
       <c r="B365" s="4" t="n">
         <v>880</v>
       </c>
-      <c r="C365" s="15" t="n">
-        <v>0</v>
+      <c r="C365" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
@@ -18583,8 +18593,10 @@
       <c r="B393" s="4" t="n">
         <v>720</v>
       </c>
-      <c r="C393" s="15" t="n">
-        <v>0</v>
+      <c r="C393" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D393" t="inlineStr">
         <is>
@@ -23707,8 +23719,10 @@
       <c r="B576" s="4" t="n">
         <v>480</v>
       </c>
-      <c r="C576" s="15" t="n">
-        <v>0</v>
+      <c r="C576" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D576" t="inlineStr">
         <is>
@@ -28747,8 +28761,10 @@
       <c r="B756" s="4" t="n">
         <v>320</v>
       </c>
-      <c r="C756" s="15" t="n">
-        <v>0</v>
+      <c r="C756" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D756" t="inlineStr">
         <is>
@@ -40003,8 +40019,10 @@
       <c r="B1158" s="4" t="n">
         <v>210</v>
       </c>
-      <c r="C1158" s="15" t="n">
-        <v>0</v>
+      <c r="C1158" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1158" t="inlineStr">
         <is>
@@ -46275,8 +46293,10 @@
       <c r="B1382" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="C1382" s="15" t="n">
-        <v>0</v>
+      <c r="C1382" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1382" t="inlineStr">
         <is>
@@ -46415,8 +46435,10 @@
       <c r="B1387" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="C1387" s="15" t="n">
-        <v>0</v>
+      <c r="C1387" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1387" t="inlineStr">
         <is>
@@ -47283,8 +47305,10 @@
       <c r="B1418" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="C1418" s="15" t="n">
-        <v>0</v>
+      <c r="C1418" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1418" t="inlineStr">
         <is>
@@ -47479,8 +47503,10 @@
       <c r="B1425" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="C1425" s="15" t="n">
-        <v>0</v>
+      <c r="C1425" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1425" t="inlineStr">
         <is>
@@ -47815,8 +47841,10 @@
       <c r="B1437" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="C1437" s="15" t="n">
-        <v>0</v>
+      <c r="C1437" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1437" t="inlineStr">
         <is>
@@ -48291,8 +48319,10 @@
       <c r="B1454" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="C1454" s="15" t="n">
-        <v>0</v>
+      <c r="C1454" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1454" t="inlineStr">
         <is>
@@ -49103,8 +49133,10 @@
       <c r="B1483" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="C1483" s="15" t="n">
-        <v>0</v>
+      <c r="C1483" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1483" t="inlineStr">
         <is>
@@ -49243,8 +49275,10 @@
       <c r="B1488" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="C1488" s="15" t="n">
-        <v>0</v>
+      <c r="C1488" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1488" t="inlineStr">
         <is>
@@ -49271,8 +49305,10 @@
       <c r="B1489" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="C1489" s="15" t="n">
-        <v>0</v>
+      <c r="C1489" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1489" t="inlineStr">
         <is>
@@ -49355,8 +49391,10 @@
       <c r="B1492" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="C1492" s="15" t="n">
-        <v>0</v>
+      <c r="C1492" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1492" t="inlineStr">
         <is>
@@ -49383,8 +49421,10 @@
       <c r="B1493" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="C1493" s="15" t="n">
-        <v>0</v>
+      <c r="C1493" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1493" t="inlineStr">
         <is>
@@ -49803,8 +49843,10 @@
       <c r="B1508" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="C1508" s="15" t="n">
-        <v>0</v>
+      <c r="C1508" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1508" t="inlineStr">
         <is>
@@ -50727,8 +50769,10 @@
       <c r="B1541" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="C1541" s="15" t="n">
-        <v>0</v>
+      <c r="C1541" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1541" t="inlineStr">
         <is>
@@ -50839,8 +50883,10 @@
       <c r="B1545" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="C1545" s="15" t="n">
-        <v>0</v>
+      <c r="C1545" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1545" t="inlineStr">
         <is>
@@ -50867,8 +50913,10 @@
       <c r="B1546" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="C1546" s="15" t="n">
-        <v>0</v>
+      <c r="C1546" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1546" t="inlineStr">
         <is>
@@ -50979,8 +51027,10 @@
       <c r="B1550" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="C1550" s="15" t="n">
-        <v>0</v>
+      <c r="C1550" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1550" t="inlineStr">
         <is>
@@ -51931,8 +51981,10 @@
       <c r="B1584" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="C1584" s="15" t="n">
-        <v>0</v>
+      <c r="C1584" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D1584" t="inlineStr">
         <is>
@@ -66080,8 +66132,10 @@
       <c r="B781" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="C781" s="15" t="n">
-        <v>0</v>
+      <c r="C781" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="D781" s="21" t="inlineStr">
         <is>
@@ -71315,7 +71369,7 @@
     <row r="17" ht="62" customHeight="1">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>Each pillar is anchored to a service you already list and a page you already own. Fibroids, myomectomy and hysterectomy is the largest at 47 articles because it holds the most unserved commercial demand. Menopause and hormone health gets 24 because your nineteen existing menopause pages are the strongest on-brand block on the site. Choosing a surgeon in Los Angeles gets 17 and carries the bottom of the funnel. Endometriosis gets 16 and PCOS 16, and those caps are deliberate: your existing pages already rank for most of those clusters, so rewriting them beats competing with them.</t>
+          <t>Each pillar is anchored to a service you already list and a page you already own. Fibroids, myomectomy and hysterectomy is the largest at 45 articles because it holds the most unserved commercial demand. Menopause and hormone health gets 25 because your nineteen existing menopause pages are the strongest on-brand block on the site. Choosing a surgeon in Los Angeles gets 17 and carries the bottom of the funnel. Endometriosis gets 17 and PCOS 16, and those caps are deliberate: your existing pages already rank for most of those clusters, so rewriting them beats competing with them.</t>
         </is>
       </c>
     </row>

</xml_diff>